<commit_message>
data: economic index update (2026-09-04 11:29 UTC)
</commit_message>
<xml_diff>
--- a/output/economic_index_latest.xlsx
+++ b/output/economic_index_latest.xlsx
@@ -681,7 +681,7 @@
         <v>0.3571428571428572</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2644239701647932</v>
+        <v>0.2644192372247186</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -690,16 +690,16 @@
         <v>100</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2161973231179675</v>
+        <v>0.2161917599160857</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>60.80986615589838</v>
+        <v>60.80958799580428</v>
       </c>
       <c r="L2" t="n">
-        <v>9.336743196911643</v>
+        <v>9.337185433532984</v>
       </c>
     </row>
   </sheetData>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>1.0005</v>
+        <v>1.0004</v>
       </c>
       <c r="O2" t="n">
         <v>4614</v>
@@ -871,7 +871,7 @@
         <v>8.452121194672523</v>
       </c>
       <c r="R2" t="n">
-        <v>1.004576741885871</v>
+        <v>1.004531044179237</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -929,19 +929,19 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>0.9983</v>
+        <v>0.9984</v>
       </c>
       <c r="O3" t="n">
-        <v>17671</v>
+        <v>17701</v>
       </c>
       <c r="P3" t="n">
         <v>36</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.783802709590148</v>
+        <v>9.78549199429842</v>
       </c>
       <c r="R3" t="n">
-        <v>1.000755233060518</v>
+        <v>1.000890629266691</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         <v>8.438799123988225</v>
       </c>
       <c r="R4" t="n">
-        <v>1.002993347368097</v>
+        <v>1.002947721689309</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -1081,7 +1081,7 @@
         <v>8.322394113111169</v>
       </c>
       <c r="R5" t="n">
-        <v>0.9891580314902595</v>
+        <v>0.9891130351732506</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         <v>8.557951183888406</v>
       </c>
       <c r="R6" t="n">
-        <v>1.017155163717697</v>
+        <v>1.017108893824781</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         <v>9.897720957641791</v>
       </c>
       <c r="R7" t="n">
-        <v>1.012407581974609</v>
+        <v>1.012369757532101</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>0.9752999999999999</v>
+        <v>0.9752</v>
       </c>
       <c r="O8" t="n">
         <v>4176</v>
@@ -1290,7 +1290,7 @@
         <v>8.358666283188001</v>
       </c>
       <c r="R8" t="n">
-        <v>0.993469159738146</v>
+        <v>0.9934239673100131</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>0.9668</v>
+        <v>0.9667</v>
       </c>
       <c r="O9" t="n">
         <v>17034</v>
@@ -1360,7 +1360,7 @@
         <v>9.745839095947058</v>
       </c>
       <c r="R9" t="n">
-        <v>0.9968720512193749</v>
+        <v>0.9968348071980339</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1417,19 +1417,19 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>0.9489</v>
+        <v>0.9488</v>
       </c>
       <c r="O10" t="n">
-        <v>250598</v>
+        <v>250602</v>
       </c>
       <c r="P10" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Q10" t="n">
-        <v>12.43370610211724</v>
+        <v>12.43372999431564</v>
       </c>
       <c r="R10" t="n">
-        <v>0.9985705529056425</v>
+        <v>0.9985177868858373</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1489,16 +1489,16 @@
         <v>0.9271</v>
       </c>
       <c r="O11" t="n">
-        <v>4804</v>
+        <v>4805</v>
       </c>
       <c r="P11" t="n">
         <v>50</v>
       </c>
       <c r="Q11" t="n">
-        <v>8.498010371999463</v>
+        <v>8.498214224818435</v>
       </c>
       <c r="R11" t="n">
-        <v>1.010030899390851</v>
+        <v>1.010009181398926</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>0.9212</v>
+        <v>0.9211</v>
       </c>
       <c r="O12" t="n">
         <v>4609</v>
@@ -1568,7 +1568,7 @@
         <v>8.443331342817782</v>
       </c>
       <c r="R12" t="n">
-        <v>1.003532024171286</v>
+        <v>1.003486373988352</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1626,7 +1626,7 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>0.9141</v>
+        <v>0.914</v>
       </c>
       <c r="O13" t="n">
         <v>4319</v>
@@ -1638,7 +1638,7 @@
         <v>8.378390788535778</v>
       </c>
       <c r="R13" t="n">
-        <v>0.9958135155348981</v>
+        <v>0.9957682164631619</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>0.907</v>
+        <v>0.9069</v>
       </c>
       <c r="O14" t="n">
         <v>4033</v>
@@ -1706,7 +1706,7 @@
         <v>8.3133619511344</v>
       </c>
       <c r="R14" t="n">
-        <v>0.9880845140096385</v>
+        <v>0.9880395665264168</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>0.8818</v>
+        <v>0.8817</v>
       </c>
       <c r="O15" t="n">
         <v>417</v>
@@ -1776,7 +1776,7 @@
         <v>6.063785208687608</v>
       </c>
       <c r="R15" t="n">
-        <v>1.01980365663123</v>
+        <v>1.019754981461143</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1790,20 +1790,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>@spotuz</t>
+          <t>@kunuzofficial</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>39787</v>
+        <v>173783</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-09-02 13:01:01</t>
+          <t>2026-09-02 16:00:12</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>trade</t>
+          <t>construction_realty</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1824,29 +1824,98 @@
         <v>0.8646647167633873</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>pos</t>
+          <t>neu</t>
         </is>
       </c>
       <c r="N16" t="n">
         <v>0.8651</v>
       </c>
       <c r="O16" t="n">
+        <v>257330</v>
+      </c>
+      <c r="P16" t="n">
+        <v>128</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>12.45911280610038</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1.000556208908821</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>**«Тўқимачи» стадиони нега бузилмоқда? Масъуллар изоҳ берди**
+Тошкент марказидаги тарихий «Тўқимачи» стадиони бузилаётгани жамоатчиликда саволлар уйғотди. Kun.uz стадионнинг мулкдори ҳамда ваколатли давлат идоралари билан боғланиб, вазиятга ойдинлик киритди.
+Қурилиш ва уй-жой коммунал хўжалиги соҳасида назорат қилиш инспекциясининг Kun.uz’га маълум қилишича, мазкур ҳудудда қурилиш-монтаж ишларини амалга ошириш учун рухсат берилган ва бу ерда автотураргоҳ, маиший хизмат кўрсатиш объекти қурилади.
+👉 https://kun.uz/kr/54488282
+[Kun.uz расмий канали](https://t.me/kunuzofficial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>@spotuz</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>39787</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-09-02 13:01:01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>trade</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>0.8646647167633873</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>0.8651</v>
+      </c>
+      <c r="O17" t="n">
         <v>4497</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>15</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>8.418035619883019</v>
       </c>
-      <c r="R16" t="n">
-        <v>1.000525501389115</v>
-      </c>
-      <c r="S16" t="inlineStr">
+      <c r="R17" t="n">
+        <v>1.000479987971438</v>
+      </c>
+      <c r="S17" t="inlineStr">
         <is>
           <t>**Часть льгот по таможенным пошлинам будет отменена с 2029 года — указ**
 Президент поручил разработать законопроект об упорядочении таможенных льгот. Бессрочно действующие льготы будут ограничены 1 января 2029 года, при этом преференции с указанием срока действия сохраняться до его конца.
@@ -1857,75 +1926,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>@kunuzofficial</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>173783</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2026-09-02 16:00:12</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>construction_realty</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="n">
-        <v>0.8646647167633873</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>0.8649</v>
-      </c>
-      <c r="O17" t="n">
-        <v>256328</v>
-      </c>
-      <c r="P17" t="n">
-        <v>128</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>12.455215272713</v>
-      </c>
-      <c r="R17" t="n">
-        <v>1.000297988329799</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>**«Тўқимачи» стадиони нега бузилмоқда? Масъуллар изоҳ берди**
-Тошкент марказидаги тарихий «Тўқимачи» стадиони бузилаётгани жамоатчиликда саволлар уйғотди. Kun.uz стадионнинг мулкдори ҳамда ваколатли давлат идоралари билан боғланиб, вазиятга ойдинлик киритди.
-Қурилиш ва уй-жой коммунал хўжалиги соҳасида назорат қилиш инспекциясининг Kun.uz’га маълум қилишича, мазкур ҳудудда қурилиш-монтаж ишларини амалга ошириш учун рухсат берилган ва бу ерда автотураргоҳ, маиший хизмат кўрсатиш объекти қурилади.
-👉 https://kun.uz/kr/54488282
-[Kun.uz расмий канали](https://t.me/kunuzofficial)</t>
-        </is>
-      </c>
-    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -1983,7 +1983,7 @@
         <v>9.759039648170255</v>
       </c>
       <c r="R18" t="n">
-        <v>0.9982222953022512</v>
+        <v>0.9981850008345972</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         <v>11.27269933367474</v>
       </c>
       <c r="R19" t="n">
-        <v>0.997542266837503</v>
+        <v>0.997493828094088</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2112,16 +2112,16 @@
         <v>0.8612</v>
       </c>
       <c r="O20" t="n">
-        <v>16805</v>
+        <v>16806</v>
       </c>
       <c r="P20" t="n">
         <v>66</v>
       </c>
       <c r="Q20" t="n">
-        <v>9.737314897481545</v>
+        <v>9.737373934586381</v>
       </c>
       <c r="R20" t="n">
-        <v>0.9960001370490649</v>
+        <v>0.99596896410235</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2178,19 +2178,19 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>0.8603</v>
+        <v>0.8605</v>
       </c>
       <c r="O21" t="n">
-        <v>16663</v>
+        <v>16693</v>
       </c>
       <c r="P21" t="n">
         <v>53</v>
       </c>
       <c r="Q21" t="n">
-        <v>9.727346854817254</v>
+        <v>9.729134165391351</v>
       </c>
       <c r="R21" t="n">
-        <v>0.9949805364749567</v>
+        <v>0.9951261748200705</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>0.8595</v>
+        <v>0.8594000000000001</v>
       </c>
       <c r="O22" t="n">
         <v>4126</v>
@@ -2260,7 +2260,7 @@
         <v>8.36287583103188</v>
       </c>
       <c r="R22" t="n">
-        <v>0.9939694854860166</v>
+        <v>0.9939242702983092</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
@@ -2327,19 +2327,19 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>0.8554</v>
+        <v>0.8552999999999999</v>
       </c>
       <c r="O23" t="n">
-        <v>15673</v>
+        <v>15674</v>
       </c>
       <c r="P23" t="n">
         <v>91</v>
       </c>
       <c r="Q23" t="n">
-        <v>9.67130325656977</v>
+        <v>9.671366322189568</v>
       </c>
       <c r="R23" t="n">
-        <v>0.9892480083475512</v>
+        <v>0.9892174997154054</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         <v>5.834810737062605</v>
       </c>
       <c r="R24" t="n">
-        <v>0.9812948712105604</v>
+        <v>0.9812480340625941</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>0.8455</v>
+        <v>0.8454</v>
       </c>
       <c r="O25" t="n">
         <v>326</v>
@@ -2485,7 +2485,7 @@
         <v>5.814130531825066</v>
       </c>
       <c r="R25" t="n">
-        <v>0.9778168870479764</v>
+        <v>0.9777702159039949</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>0.7935</v>
+        <v>0.7934</v>
       </c>
       <c r="O26" t="n">
         <v>413</v>
@@ -2553,7 +2553,7 @@
         <v>6.073044534100405</v>
       </c>
       <c r="R26" t="n">
-        <v>1.021360884268578</v>
+        <v>1.021312134772104</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -2612,16 +2612,16 @@
         <v>0.7801</v>
       </c>
       <c r="O27" t="n">
-        <v>84567</v>
+        <v>84568</v>
       </c>
       <c r="P27" t="n">
         <v>90</v>
       </c>
       <c r="Q27" t="n">
-        <v>11.34743742614418</v>
+        <v>11.34744922576305</v>
       </c>
       <c r="R27" t="n">
-        <v>1.004155980551871</v>
+        <v>1.004108264778836</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -2680,16 +2680,16 @@
         <v>0.7793</v>
       </c>
       <c r="O28" t="n">
-        <v>265451</v>
+        <v>265452</v>
       </c>
       <c r="P28" t="n">
         <v>217</v>
       </c>
       <c r="Q28" t="n">
-        <v>12.49082292447228</v>
+        <v>12.49082668547557</v>
       </c>
       <c r="R28" t="n">
-        <v>1.00315769501845</v>
+        <v>1.003103061113409</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         <v>9.803722464346553</v>
       </c>
       <c r="R29" t="n">
-        <v>1.002792763804491</v>
+        <v>1.002755298580092</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
@@ -2817,16 +2817,16 @@
         <v>0.7771</v>
       </c>
       <c r="O30" t="n">
-        <v>81067</v>
+        <v>81068</v>
       </c>
       <c r="P30" t="n">
         <v>24</v>
       </c>
       <c r="Q30" t="n">
-        <v>11.30363550794455</v>
+        <v>11.30364783589263</v>
       </c>
       <c r="R30" t="n">
-        <v>1.000279866812001</v>
+        <v>1.0002323860062</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -2882,19 +2882,19 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>0.7764</v>
+        <v>0.7765</v>
       </c>
       <c r="O31" t="n">
-        <v>17448</v>
+        <v>17478</v>
       </c>
       <c r="P31" t="n">
         <v>31</v>
       </c>
       <c r="Q31" t="n">
-        <v>9.770584533871901</v>
+        <v>9.772296276843781</v>
       </c>
       <c r="R31" t="n">
-        <v>0.9994031863242749</v>
+        <v>0.9995409301453289</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -2954,16 +2954,16 @@
         <v>0.7754</v>
       </c>
       <c r="O32" t="n">
-        <v>79116</v>
+        <v>79117</v>
       </c>
       <c r="P32" t="n">
         <v>14</v>
       </c>
       <c r="Q32" t="n">
-        <v>11.27903689211984</v>
+        <v>11.27904952707697</v>
       </c>
       <c r="R32" t="n">
-        <v>0.9981030892483919</v>
+        <v>0.9980557413092315</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="N33" t="n">
-        <v>0.7744</v>
+        <v>0.7743</v>
       </c>
       <c r="O33" t="n">
         <v>366</v>
@@ -3031,7 +3031,7 @@
         <v>5.926926025970411</v>
       </c>
       <c r="R33" t="n">
-        <v>0.9967867636880899</v>
+        <v>0.9967391871129835</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -3090,16 +3090,16 @@
         <v>0.7739</v>
       </c>
       <c r="O34" t="n">
-        <v>243544</v>
+        <v>243545</v>
       </c>
       <c r="P34" t="n">
         <v>127</v>
       </c>
       <c r="Q34" t="n">
-        <v>12.40409939429817</v>
+        <v>12.40410349602931</v>
       </c>
       <c r="R34" t="n">
-        <v>0.9961927914921277</v>
+        <v>0.9961385663691004</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
         <v>8.310414994188292</v>
       </c>
       <c r="R35" t="n">
-        <v>0.9877342534845924</v>
+        <v>0.9876893219345514</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         <v>8.299285906897275</v>
       </c>
       <c r="R36" t="n">
-        <v>0.9864115059761893</v>
+        <v>0.9863666345972881</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="N37" t="n">
-        <v>0.7557</v>
+        <v>0.7556</v>
       </c>
       <c r="O37" t="n">
         <v>318</v>
@@ -3307,7 +3307,7 @@
         <v>5.783825182329737</v>
       </c>
       <c r="R37" t="n">
-        <v>0.9727201520603082</v>
+        <v>0.9726737241831955</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -3363,19 +3363,19 @@
         </is>
       </c>
       <c r="N38" t="n">
-        <v>0.6424</v>
+        <v>0.6425999999999999</v>
       </c>
       <c r="O38" t="n">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="P38" t="n">
         <v>3</v>
       </c>
       <c r="Q38" t="n">
-        <v>6.042632833682381</v>
+        <v>6.045005314036012</v>
       </c>
       <c r="R38" t="n">
-        <v>1.016246263248321</v>
+        <v>1.016596741110735</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
@@ -3434,16 +3434,16 @@
         <v>0.6334</v>
       </c>
       <c r="O39" t="n">
-        <v>82597</v>
+        <v>82598</v>
       </c>
       <c r="P39" t="n">
         <v>93</v>
       </c>
       <c r="Q39" t="n">
-        <v>11.32399008498576</v>
+        <v>11.32400216454171</v>
       </c>
       <c r="R39" t="n">
-        <v>1.0020810814387</v>
+        <v>1.002033491189748</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -3499,19 +3499,19 @@
         </is>
       </c>
       <c r="N40" t="n">
-        <v>0.6332</v>
+        <v>0.6333</v>
       </c>
       <c r="O40" t="n">
-        <v>17848</v>
+        <v>17878</v>
       </c>
       <c r="P40" t="n">
         <v>27</v>
       </c>
       <c r="Q40" t="n">
-        <v>9.792723575551273</v>
+        <v>9.794397869948424</v>
       </c>
       <c r="R40" t="n">
-        <v>1.001667721134841</v>
+        <v>1.001801549993896</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
@@ -3571,16 +3571,16 @@
         <v>0.6321</v>
       </c>
       <c r="O41" t="n">
-        <v>255668</v>
+        <v>255669</v>
       </c>
       <c r="P41" t="n">
         <v>48</v>
       </c>
       <c r="Q41" t="n">
-        <v>12.45201433312036</v>
+        <v>12.45201824295183</v>
       </c>
       <c r="R41" t="n">
-        <v>1.000040915821202</v>
+        <v>0.9999864645523602</v>
       </c>
       <c r="S41" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="N42" t="n">
-        <v>0.6321</v>
+        <v>0.632</v>
       </c>
       <c r="O42" t="n">
         <v>363</v>
@@ -3655,7 +3655,7 @@
         <v>5.945420608606575</v>
       </c>
       <c r="R42" t="n">
-        <v>0.9998971711895309</v>
+        <v>0.9998494461548528</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
@@ -3711,19 +3711,19 @@
         </is>
       </c>
       <c r="N43" t="n">
-        <v>0.6317</v>
+        <v>0.6316000000000001</v>
       </c>
       <c r="O43" t="n">
-        <v>253225</v>
+        <v>253226</v>
       </c>
       <c r="P43" t="n">
         <v>71</v>
       </c>
       <c r="Q43" t="n">
-        <v>12.44259825633764</v>
+        <v>12.44260220315818</v>
       </c>
       <c r="R43" t="n">
-        <v>0.9992846958396531</v>
+        <v>0.9992302889541865</v>
       </c>
       <c r="S43" t="inlineStr">
         <is>
@@ -3781,19 +3781,19 @@
         </is>
       </c>
       <c r="N44" t="n">
-        <v>0.6316000000000001</v>
+        <v>0.6315</v>
       </c>
       <c r="O44" t="n">
-        <v>252188</v>
+        <v>252190</v>
       </c>
       <c r="P44" t="n">
         <v>314</v>
       </c>
       <c r="Q44" t="n">
-        <v>12.44042118582932</v>
+        <v>12.44042909665845</v>
       </c>
       <c r="R44" t="n">
-        <v>0.9991098518725078</v>
+        <v>0.999055772900374</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
@@ -3854,16 +3854,16 @@
         <v>0.6314</v>
       </c>
       <c r="O45" t="n">
-        <v>79741</v>
+        <v>79742</v>
       </c>
       <c r="P45" t="n">
         <v>36</v>
       </c>
       <c r="Q45" t="n">
-        <v>11.28745420664684</v>
+        <v>11.28746673569858</v>
       </c>
       <c r="R45" t="n">
-        <v>0.9988479531683286</v>
+        <v>0.9988005596886901</v>
       </c>
       <c r="S45" t="inlineStr">
         <is>
@@ -3931,7 +3931,7 @@
         <v>9.734180932819669</v>
       </c>
       <c r="R46" t="n">
-        <v>0.9956795733961894</v>
+        <v>0.9956423739268743</v>
       </c>
       <c r="S46" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
         <v>5.905361848054571</v>
       </c>
       <c r="R47" t="n">
-        <v>0.9931601135456487</v>
+        <v>0.9931127100703457</v>
       </c>
       <c r="S47" t="inlineStr">
         <is>
@@ -4068,7 +4068,7 @@
         <v>5.902633333401366</v>
       </c>
       <c r="R48" t="n">
-        <v>0.9927012336340509</v>
+        <v>0.9926538520610599</v>
       </c>
       <c r="S48" t="inlineStr">
         <is>
@@ -4136,7 +4136,7 @@
         <v>5.902633333401366</v>
       </c>
       <c r="R49" t="n">
-        <v>0.9927012336340509</v>
+        <v>0.9926538520610599</v>
       </c>
       <c r="S49" t="inlineStr">
         <is>
@@ -4195,16 +4195,16 @@
         <v>0.6267</v>
       </c>
       <c r="O50" t="n">
-        <v>229564</v>
+        <v>229565</v>
       </c>
       <c r="P50" t="n">
         <v>175</v>
       </c>
       <c r="Q50" t="n">
-        <v>12.34546495438189</v>
+        <v>12.34546930380591</v>
       </c>
       <c r="R50" t="n">
-        <v>0.9914837671187312</v>
+        <v>0.9914298197675971</v>
       </c>
       <c r="S50" t="inlineStr">
         <is>
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="N51" t="n">
-        <v>0.6194</v>
+        <v>0.6193</v>
       </c>
       <c r="O51" t="n">
         <v>330</v>
@@ -4274,7 +4274,7 @@
         <v>5.82600010738045</v>
       </c>
       <c r="R51" t="n">
-        <v>0.9798131049444644</v>
+        <v>0.9797663385211171</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -4342,7 +4342,7 @@
         <v>5.820082930352362</v>
       </c>
       <c r="R52" t="n">
-        <v>0.9788179577612275</v>
+        <v>0.9787712388361982</v>
       </c>
       <c r="S52" t="inlineStr">
         <is>
@@ -4410,7 +4410,7 @@
         <v>6.049733455231958</v>
       </c>
       <c r="R53" t="n">
-        <v>1.017440441401307</v>
+        <v>1.017391879027347</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
@@ -4469,16 +4469,16 @@
         <v>0.6326000000000001</v>
       </c>
       <c r="O54" t="n">
-        <v>81566</v>
+        <v>81567</v>
       </c>
       <c r="P54" t="n">
         <v>2</v>
       </c>
       <c r="Q54" t="n">
-        <v>11.30922908562858</v>
+        <v>11.30924134481224</v>
       </c>
       <c r="R54" t="n">
-        <v>1.00077485297259</v>
+        <v>1.000727342046413</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
@@ -4534,7 +4534,7 @@
         </is>
       </c>
       <c r="N55" t="n">
-        <v>0.6324</v>
+        <v>0.6323</v>
       </c>
       <c r="O55" t="n">
         <v>4500</v>
@@ -4546,7 +4546,7 @@
         <v>8.416930769477844</v>
       </c>
       <c r="R55" t="n">
-        <v>1.000394184410248</v>
+        <v>1.000348676966116</v>
       </c>
       <c r="S55" t="inlineStr">
         <is>
@@ -4601,19 +4601,19 @@
         </is>
       </c>
       <c r="N56" t="n">
-        <v>0.6291</v>
+        <v>0.6292</v>
       </c>
       <c r="O56" t="n">
-        <v>16802</v>
+        <v>16832</v>
       </c>
       <c r="P56" t="n">
         <v>7</v>
       </c>
       <c r="Q56" t="n">
-        <v>9.73014555852275</v>
+        <v>9.731927878386204</v>
       </c>
       <c r="R56" t="n">
-        <v>0.9952668073107653</v>
+        <v>0.9954119244951035</v>
       </c>
       <c r="S56" t="inlineStr">
         <is>
@@ -4671,16 +4671,16 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>81850</v>
+        <v>81851</v>
       </c>
       <c r="P57" t="n">
         <v>32</v>
       </c>
       <c r="Q57" t="n">
-        <v>11.31343740325436</v>
+        <v>11.3134496109562</v>
       </c>
       <c r="R57" t="n">
-        <v>1.001147254877381</v>
+        <v>1.001099721312579</v>
       </c>
       <c r="S57" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="O58" t="n">
-        <v>83556</v>
+        <v>83857</v>
       </c>
       <c r="P58" t="n">
         <v>19</v>
       </c>
       <c r="Q58" t="n">
-        <v>11.33373898867175</v>
+        <v>11.33733321551424</v>
       </c>
       <c r="R58" t="n">
-        <v>1.002943780176087</v>
+        <v>1.003213123562926</v>
       </c>
       <c r="S58" t="inlineStr">
         <is>
@@ -4807,16 +4807,16 @@
         <v>0</v>
       </c>
       <c r="O59" t="n">
-        <v>80449</v>
+        <v>80450</v>
       </c>
       <c r="P59" t="n">
         <v>2</v>
       </c>
       <c r="Q59" t="n">
-        <v>11.2954408715077</v>
+        <v>11.29545330089325</v>
       </c>
       <c r="R59" t="n">
-        <v>0.9995547080931203</v>
+        <v>0.999507271475596</v>
       </c>
       <c r="S59" t="inlineStr">
         <is>
@@ -4875,16 +4875,16 @@
         <v>0</v>
       </c>
       <c r="O60" t="n">
-        <v>83364</v>
+        <v>83365</v>
       </c>
       <c r="P60" t="n">
         <v>55</v>
       </c>
       <c r="Q60" t="n">
-        <v>11.33230246481186</v>
+        <v>11.33231444437472</v>
       </c>
       <c r="R60" t="n">
-        <v>1.002816659490513</v>
+        <v>1.002769024675153</v>
       </c>
       <c r="S60" t="inlineStr">
         <is>
@@ -4943,16 +4943,16 @@
         <v>0</v>
       </c>
       <c r="O61" t="n">
-        <v>80660</v>
+        <v>80661</v>
       </c>
       <c r="P61" t="n">
         <v>15</v>
       </c>
       <c r="Q61" t="n">
-        <v>11.29838232387519</v>
+        <v>11.29839471675424</v>
       </c>
       <c r="R61" t="n">
-        <v>0.9998150027195988</v>
+        <v>0.9997675502322938</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
@@ -5011,16 +5011,16 @@
         <v>0</v>
       </c>
       <c r="O62" t="n">
-        <v>80243</v>
+        <v>80244</v>
       </c>
       <c r="P62" t="n">
         <v>12</v>
       </c>
       <c r="Q62" t="n">
-        <v>11.29312631490641</v>
+        <v>11.29313877309362</v>
       </c>
       <c r="R62" t="n">
-        <v>0.999349888646559</v>
+        <v>0.999302464523264</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
@@ -5079,16 +5079,16 @@
         <v>0</v>
       </c>
       <c r="O63" t="n">
-        <v>80659</v>
+        <v>80960</v>
       </c>
       <c r="P63" t="n">
         <v>55</v>
       </c>
       <c r="Q63" t="n">
-        <v>11.29936088843634</v>
+        <v>11.3030805929248</v>
       </c>
       <c r="R63" t="n">
-        <v>0.9999015977295146</v>
+        <v>1.000182192051523</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -5147,16 +5147,16 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>80433</v>
+        <v>80734</v>
       </c>
       <c r="P64" t="n">
         <v>22</v>
       </c>
       <c r="Q64" t="n">
-        <v>11.29573913413014</v>
+        <v>11.29947230973897</v>
       </c>
       <c r="R64" t="n">
-        <v>0.9995811019109364</v>
+        <v>0.9998629038223834</v>
       </c>
       <c r="S64" t="inlineStr">
         <is>
@@ -5215,16 +5215,16 @@
         <v>0</v>
       </c>
       <c r="O65" t="n">
-        <v>81113</v>
+        <v>81114</v>
       </c>
       <c r="P65" t="n">
         <v>11</v>
       </c>
       <c r="Q65" t="n">
-        <v>11.3038820380348</v>
+        <v>11.30389436294406</v>
       </c>
       <c r="R65" t="n">
-        <v>1.000301682721198</v>
+        <v>1.000254200587161</v>
       </c>
       <c r="S65" t="inlineStr">
         <is>
@@ -5283,16 +5283,16 @@
         <v>0</v>
       </c>
       <c r="O66" t="n">
-        <v>81485</v>
+        <v>81486</v>
       </c>
       <c r="P66" t="n">
         <v>21</v>
       </c>
       <c r="Q66" t="n">
-        <v>11.30870179850853</v>
+        <v>11.30871406415796</v>
       </c>
       <c r="R66" t="n">
-        <v>1.000728192348241</v>
+        <v>1.000680684259955</v>
       </c>
       <c r="S66" t="inlineStr">
         <is>
@@ -5351,16 +5351,16 @@
         <v>0</v>
       </c>
       <c r="O67" t="n">
-        <v>81221</v>
+        <v>81222</v>
       </c>
       <c r="P67" t="n">
         <v>43</v>
       </c>
       <c r="Q67" t="n">
-        <v>11.30599969167885</v>
+        <v>11.306011990516</v>
       </c>
       <c r="R67" t="n">
-        <v>1.000489077856465</v>
+        <v>1.000441584315821</v>
       </c>
       <c r="S67" t="inlineStr">
         <is>
@@ -5419,16 +5419,16 @@
         <v>0</v>
       </c>
       <c r="O68" t="n">
-        <v>81352</v>
+        <v>81353</v>
       </c>
       <c r="P68" t="n">
         <v>11</v>
       </c>
       <c r="Q68" t="n">
-        <v>11.30682337951087</v>
+        <v>11.30683566822185</v>
       </c>
       <c r="R68" t="n">
-        <v>1.000561967534687</v>
+        <v>1.000514469558619</v>
       </c>
       <c r="S68" t="inlineStr">
         <is>
@@ -5487,16 +5487,16 @@
         <v>0</v>
       </c>
       <c r="O69" t="n">
-        <v>79925</v>
+        <v>79926</v>
       </c>
       <c r="P69" t="n">
         <v>1</v>
       </c>
       <c r="Q69" t="n">
-        <v>11.28888150841285</v>
+        <v>11.28889401959472</v>
       </c>
       <c r="R69" t="n">
-        <v>0.9989742577735511</v>
+        <v>0.9989268565795411</v>
       </c>
       <c r="S69" t="inlineStr">
         <is>
@@ -5555,16 +5555,16 @@
         <v>0</v>
       </c>
       <c r="O70" t="n">
-        <v>79534</v>
+        <v>79535</v>
       </c>
       <c r="P70" t="n">
         <v>30</v>
       </c>
       <c r="Q70" t="n">
-        <v>11.28470655578924</v>
+        <v>11.28471911931356</v>
       </c>
       <c r="R70" t="n">
-        <v>0.9986048084002619</v>
+        <v>0.998557429777663</v>
       </c>
       <c r="S70" t="inlineStr">
         <is>
@@ -5623,16 +5623,16 @@
         <v>0</v>
       </c>
       <c r="O71" t="n">
-        <v>79952</v>
+        <v>79953</v>
       </c>
       <c r="P71" t="n">
         <v>27</v>
       </c>
       <c r="Q71" t="n">
-        <v>11.28986940982812</v>
+        <v>11.28988190865635</v>
       </c>
       <c r="R71" t="n">
-        <v>0.9990616790191661</v>
+        <v>0.9990142724870045</v>
       </c>
       <c r="S71" t="inlineStr">
         <is>
@@ -5691,16 +5691,16 @@
         <v>0</v>
       </c>
       <c r="O72" t="n">
-        <v>81935</v>
+        <v>81936</v>
       </c>
       <c r="P72" t="n">
         <v>33</v>
       </c>
       <c r="Q72" t="n">
-        <v>11.31449891619286</v>
+        <v>11.31451111094302</v>
       </c>
       <c r="R72" t="n">
-        <v>1.001241190144489</v>
+        <v>1.001193650872307</v>
       </c>
       <c r="S72" t="inlineStr">
         <is>
@@ -5759,16 +5759,16 @@
         <v>0</v>
       </c>
       <c r="O73" t="n">
-        <v>80628</v>
+        <v>80629</v>
       </c>
       <c r="P73" t="n">
         <v>60</v>
       </c>
       <c r="Q73" t="n">
-        <v>11.29910085710729</v>
+        <v>11.2991132410849</v>
       </c>
       <c r="R73" t="n">
-        <v>0.9998785870704214</v>
+        <v>0.9998311307079151</v>
       </c>
       <c r="S73" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         <v>11.26009560328566</v>
       </c>
       <c r="R74" t="n">
-        <v>0.9964269391408458</v>
+        <v>0.9963785545556093</v>
       </c>
       <c r="S74" t="inlineStr">
         <is>
@@ -5895,16 +5895,16 @@
         <v>0</v>
       </c>
       <c r="O75" t="n">
-        <v>78497</v>
+        <v>78498</v>
       </c>
       <c r="P75" t="n">
         <v>35</v>
       </c>
       <c r="Q75" t="n">
-        <v>11.27171977083761</v>
+        <v>11.27173249858474</v>
       </c>
       <c r="R75" t="n">
-        <v>0.9974555834882768</v>
+        <v>0.9974082752015182</v>
       </c>
       <c r="S75" t="inlineStr">
         <is>
@@ -5963,16 +5963,16 @@
         <v>0</v>
       </c>
       <c r="O76" t="n">
-        <v>80774</v>
+        <v>80775</v>
       </c>
       <c r="P76" t="n">
         <v>28</v>
       </c>
       <c r="Q76" t="n">
-        <v>11.30011583429555</v>
+        <v>11.30012820571016</v>
       </c>
       <c r="R76" t="n">
-        <v>0.9999684043018755</v>
+        <v>0.9999209424663469</v>
       </c>
       <c r="S76" t="inlineStr">
         <is>
@@ -6031,16 +6031,16 @@
         <v>0</v>
       </c>
       <c r="O77" t="n">
-        <v>81915</v>
+        <v>82216</v>
       </c>
       <c r="P77" t="n">
         <v>13</v>
       </c>
       <c r="Q77" t="n">
-        <v>11.31376695890648</v>
+        <v>11.31743355862289</v>
       </c>
       <c r="R77" t="n">
-        <v>1.001176417873974</v>
+        <v>1.001452251180655</v>
       </c>
       <c r="S77" t="inlineStr">
         <is>
@@ -6099,16 +6099,16 @@
         <v>0</v>
       </c>
       <c r="O78" t="n">
-        <v>81510</v>
+        <v>81810</v>
       </c>
       <c r="P78" t="n">
         <v>14</v>
       </c>
       <c r="Q78" t="n">
-        <v>11.30883671237849</v>
+        <v>11.31250918158702</v>
       </c>
       <c r="R78" t="n">
-        <v>1.000740131129157</v>
+        <v>1.001016504998212</v>
       </c>
       <c r="S78" t="inlineStr">
         <is>
@@ -6176,7 +6176,7 @@
         <v>11.29151790594907</v>
       </c>
       <c r="R79" t="n">
-        <v>0.9992075575269387</v>
+        <v>0.9991590379201948</v>
       </c>
       <c r="S79" t="inlineStr">
         <is>
@@ -6244,7 +6244,7 @@
         <v>11.29603730781853</v>
       </c>
       <c r="R80" t="n">
-        <v>0.9996074878588106</v>
+        <v>0.9995589488322152</v>
       </c>
       <c r="S80" t="inlineStr">
         <is>
@@ -6312,7 +6312,7 @@
         <v>11.28838093274039</v>
       </c>
       <c r="R81" t="n">
-        <v>0.9989299608952034</v>
+        <v>0.9988814547680206</v>
       </c>
       <c r="S81" t="inlineStr">
         <is>
@@ -6380,7 +6380,7 @@
         <v>11.28269435615412</v>
       </c>
       <c r="R82" t="n">
-        <v>0.9984267450876582</v>
+        <v>0.998378263395672</v>
       </c>
       <c r="S82" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
         <v>11.31543747709451</v>
       </c>
       <c r="R83" t="n">
-        <v>1.001324245155689</v>
+        <v>1.001275622766644</v>
       </c>
       <c r="S83" t="inlineStr">
         <is>
@@ -6521,7 +6521,7 @@
         <v>9.906881785604144</v>
       </c>
       <c r="R84" t="n">
-        <v>1.013344615027565</v>
+        <v>1.013306755576674</v>
       </c>
       <c r="S84" t="inlineStr">
         <is>
@@ -6589,7 +6589,7 @@
         <v>9.940638818166921</v>
       </c>
       <c r="R85" t="n">
-        <v>1.016797518565438</v>
+        <v>1.016759530111017</v>
       </c>
       <c r="S85" t="inlineStr">
         <is>
@@ -6657,7 +6657,7 @@
         <v>9.838095333769076</v>
       </c>
       <c r="R86" t="n">
-        <v>1.006308659409804</v>
+        <v>1.006271062828436</v>
       </c>
       <c r="S86" t="inlineStr">
         <is>
@@ -6725,7 +6725,7 @@
         <v>9.777470711952642</v>
       </c>
       <c r="R87" t="n">
-        <v>1.000107552403053</v>
+        <v>1.000070187500526</v>
       </c>
       <c r="S87" t="inlineStr">
         <is>
@@ -6784,16 +6784,16 @@
         <v>0</v>
       </c>
       <c r="O88" t="n">
-        <v>17101</v>
+        <v>17102</v>
       </c>
       <c r="P88" t="n">
         <v>24</v>
       </c>
       <c r="Q88" t="n">
-        <v>9.749753452594087</v>
+        <v>9.749811759932081</v>
       </c>
       <c r="R88" t="n">
-        <v>0.9972724387798005</v>
+        <v>0.9972411436559402</v>
       </c>
       <c r="S88" t="inlineStr">
         <is>
@@ -6852,16 +6852,16 @@
         <v>0</v>
       </c>
       <c r="O89" t="n">
-        <v>16513</v>
+        <v>16514</v>
       </c>
       <c r="P89" t="n">
         <v>37</v>
       </c>
       <c r="Q89" t="n">
-        <v>9.716434821366272</v>
+        <v>9.716495104092274</v>
       </c>
       <c r="R89" t="n">
-        <v>0.9938643779726294</v>
+        <v>0.9938334122257786</v>
       </c>
       <c r="S89" t="inlineStr">
         <is>
@@ -6931,7 +6931,7 @@
         <v>9.742496866444002</v>
       </c>
       <c r="R90" t="n">
-        <v>0.9965301847933487</v>
+        <v>0.9964929535444396</v>
       </c>
       <c r="S90" t="inlineStr">
         <is>
@@ -7000,7 +7000,7 @@
         <v>9.740497924041666</v>
       </c>
       <c r="R91" t="n">
-        <v>0.996325719093344</v>
+        <v>0.9962884954834542</v>
       </c>
       <c r="S91" t="inlineStr">
         <is>
@@ -7068,7 +7068,7 @@
         <v>9.749986661550366</v>
       </c>
       <c r="R92" t="n">
-        <v>0.9972962930101362</v>
+        <v>0.9972590331387468</v>
       </c>
       <c r="S92" t="inlineStr">
         <is>
@@ -7136,7 +7136,7 @@
         <v>9.756146964637418</v>
       </c>
       <c r="R93" t="n">
-        <v>0.9979264115575558</v>
+        <v>0.9978891281443801</v>
       </c>
       <c r="S93" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
         <v>9.762499859235151</v>
       </c>
       <c r="R94" t="n">
-        <v>0.9985762297011218</v>
+        <v>0.9985389220101657</v>
       </c>
       <c r="S94" t="inlineStr">
         <is>
@@ -7274,7 +7274,7 @@
         <v>9.751617603198001</v>
       </c>
       <c r="R95" t="n">
-        <v>0.9974631170393132</v>
+        <v>0.9974258509352305</v>
       </c>
       <c r="S95" t="inlineStr">
         <is>
@@ -7341,7 +7341,7 @@
         <v>9.801676286389442</v>
       </c>
       <c r="R96" t="n">
-        <v>1.002583466524166</v>
+        <v>1.002546009119299</v>
       </c>
       <c r="S96" t="inlineStr">
         <is>
@@ -7410,7 +7410,7 @@
         <v>9.739438040529622</v>
       </c>
       <c r="R97" t="n">
-        <v>0.9962173068529712</v>
+        <v>0.9961800872934585</v>
       </c>
       <c r="S97" t="inlineStr">
         <is>
@@ -7478,7 +7478,7 @@
         <v>9.734240155229445</v>
       </c>
       <c r="R98" t="n">
-        <v>0.9956856310752185</v>
+        <v>0.995648431379583</v>
       </c>
       <c r="S98" t="inlineStr">
         <is>
@@ -7537,16 +7537,16 @@
         <v>0</v>
       </c>
       <c r="O99" t="n">
-        <v>17335</v>
+        <v>17365</v>
       </c>
       <c r="P99" t="n">
         <v>111</v>
       </c>
       <c r="Q99" t="n">
-        <v>9.773264965486154</v>
+        <v>9.7749721303007</v>
       </c>
       <c r="R99" t="n">
-        <v>0.9996773594698757</v>
+        <v>0.999814624779373</v>
       </c>
       <c r="S99" t="inlineStr">
         <is>
@@ -7614,7 +7614,7 @@
         <v>9.881293067026359</v>
       </c>
       <c r="R100" t="n">
-        <v>1.010727223325775</v>
+        <v>1.010689461662952</v>
       </c>
       <c r="S100" t="inlineStr">
         <is>
@@ -7674,16 +7674,16 @@
         <v>0</v>
       </c>
       <c r="O101" t="n">
-        <v>289570</v>
+        <v>290572</v>
       </c>
       <c r="P101" t="n">
         <v>70</v>
       </c>
       <c r="Q101" t="n">
-        <v>12.57663915335071</v>
+        <v>12.58009180518932</v>
       </c>
       <c r="R101" t="n">
-        <v>1.010049731746326</v>
+        <v>1.010271691108062</v>
       </c>
       <c r="S101" t="inlineStr">
         <is>
@@ -7743,16 +7743,16 @@
         <v>0</v>
       </c>
       <c r="O102" t="n">
-        <v>274477</v>
+        <v>274479</v>
       </c>
       <c r="P102" t="n">
         <v>1224</v>
       </c>
       <c r="Q102" t="n">
-        <v>12.53150560146465</v>
+        <v>12.53151282358456</v>
       </c>
       <c r="R102" t="n">
-        <v>1.006424984990104</v>
+        <v>1.006370450110925</v>
       </c>
       <c r="S102" t="inlineStr">
         <is>
@@ -7811,16 +7811,16 @@
         <v>0</v>
       </c>
       <c r="O103" t="n">
-        <v>265240</v>
+        <v>265241</v>
       </c>
       <c r="P103" t="n">
         <v>370</v>
       </c>
       <c r="Q103" t="n">
-        <v>12.49118015664127</v>
+        <v>12.49118391630124</v>
       </c>
       <c r="R103" t="n">
-        <v>1.003186384897523</v>
+        <v>1.00313174931346</v>
       </c>
       <c r="S103" t="inlineStr">
         <is>
@@ -7880,16 +7880,16 @@
         <v>0</v>
       </c>
       <c r="O104" t="n">
-        <v>269689</v>
+        <v>269690</v>
       </c>
       <c r="P104" t="n">
         <v>190</v>
       </c>
       <c r="Q104" t="n">
-        <v>12.5064364636379</v>
+        <v>12.50644016637477</v>
       </c>
       <c r="R104" t="n">
-        <v>1.004411642981299</v>
+        <v>1.004356935727076</v>
       </c>
       <c r="S104" t="inlineStr">
         <is>
@@ -7949,16 +7949,16 @@
         <v>0</v>
       </c>
       <c r="O105" t="n">
-        <v>251575</v>
+        <v>251577</v>
       </c>
       <c r="P105" t="n">
         <v>187</v>
       </c>
       <c r="Q105" t="n">
-        <v>12.43698593410874</v>
+        <v>12.43699387216019</v>
       </c>
       <c r="R105" t="n">
-        <v>0.9988339613872568</v>
+        <v>0.998779899709865</v>
       </c>
       <c r="S105" t="inlineStr">
         <is>
@@ -8017,16 +8017,16 @@
         <v>0</v>
       </c>
       <c r="O106" t="n">
-        <v>259816</v>
+        <v>259817</v>
       </c>
       <c r="P106" t="n">
         <v>36</v>
       </c>
       <c r="Q106" t="n">
-        <v>12.46800989576314</v>
+        <v>12.4680137435523</v>
       </c>
       <c r="R106" t="n">
-        <v>1.001325544692196</v>
+        <v>1.00127101809076</v>
       </c>
       <c r="S106" t="inlineStr">
         <is>
@@ -8086,16 +8086,16 @@
         <v>0</v>
       </c>
       <c r="O107" t="n">
-        <v>262016</v>
+        <v>262017</v>
       </c>
       <c r="P107" t="n">
         <v>83</v>
       </c>
       <c r="Q107" t="n">
-        <v>12.47679801220674</v>
+        <v>12.47680182632929</v>
       </c>
       <c r="R107" t="n">
-        <v>1.002031332188218</v>
+        <v>1.001976764232061</v>
       </c>
       <c r="S107" t="inlineStr">
         <is>
@@ -8155,16 +8155,16 @@
         <v>0</v>
       </c>
       <c r="O108" t="n">
-        <v>250996</v>
+        <v>250997</v>
       </c>
       <c r="P108" t="n">
         <v>162</v>
       </c>
       <c r="Q108" t="n">
-        <v>12.4344862854999</v>
+        <v>12.43449026446707</v>
       </c>
       <c r="R108" t="n">
-        <v>0.9986332106639482</v>
+        <v>0.9985788420373803</v>
       </c>
       <c r="S108" t="inlineStr">
         <is>
@@ -8223,16 +8223,16 @@
         <v>0</v>
       </c>
       <c r="O109" t="n">
-        <v>249491</v>
+        <v>249492</v>
       </c>
       <c r="P109" t="n">
         <v>102</v>
       </c>
       <c r="Q109" t="n">
-        <v>12.42799945691649</v>
+        <v>12.42800346177839</v>
       </c>
       <c r="R109" t="n">
-        <v>0.9981122432265697</v>
+        <v>0.9980579052092819</v>
       </c>
       <c r="S109" t="inlineStr">
         <is>
@@ -8296,16 +8296,16 @@
         <v>0</v>
       </c>
       <c r="O110" t="n">
-        <v>253587</v>
+        <v>254588</v>
       </c>
       <c r="P110" t="n">
         <v>758</v>
       </c>
       <c r="Q110" t="n">
-        <v>12.44942658413241</v>
+        <v>12.45334279562062</v>
       </c>
       <c r="R110" t="n">
-        <v>0.9998330896174572</v>
+        <v>1.00009283564133</v>
       </c>
       <c r="S110" t="inlineStr">
         <is>
@@ -8372,16 +8372,16 @@
         <v>0</v>
       </c>
       <c r="O111" t="n">
-        <v>236845</v>
+        <v>236846</v>
       </c>
       <c r="P111" t="n">
         <v>34</v>
       </c>
       <c r="Q111" t="n">
-        <v>12.375452485066</v>
+        <v>12.37545670599802</v>
       </c>
       <c r="R111" t="n">
-        <v>0.9938921130173373</v>
+        <v>0.9938380234590886</v>
       </c>
       <c r="S111" t="inlineStr">
         <is>
@@ -8440,16 +8440,16 @@
         <v>0</v>
       </c>
       <c r="O112" t="n">
-        <v>260801</v>
+        <v>261803</v>
       </c>
       <c r="P112" t="n">
         <v>1391</v>
       </c>
       <c r="Q112" t="n">
-        <v>12.48212738174098</v>
+        <v>12.4859216192103</v>
       </c>
       <c r="R112" t="n">
-        <v>1.00245934226331</v>
+        <v>1.002709149076235</v>
       </c>
       <c r="S112" t="inlineStr">
         <is>
@@ -8508,16 +8508,16 @@
         <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>248585</v>
+        <v>248586</v>
       </c>
       <c r="P113" t="n">
         <v>239</v>
       </c>
       <c r="Q113" t="n">
-        <v>12.42546517053323</v>
+        <v>12.42546918555745</v>
       </c>
       <c r="R113" t="n">
-        <v>0.9979087106889521</v>
+        <v>0.9978543846338273</v>
       </c>
       <c r="S113" t="inlineStr">
         <is>
@@ -8576,16 +8576,16 @@
         <v>0</v>
       </c>
       <c r="O114" t="n">
-        <v>243605</v>
+        <v>243606</v>
       </c>
       <c r="P114" t="n">
         <v>156</v>
       </c>
       <c r="Q114" t="n">
-        <v>12.40458738221888</v>
+        <v>12.40459148194891</v>
       </c>
       <c r="R114" t="n">
-        <v>0.9962319825719061</v>
+        <v>0.9961777551419543</v>
       </c>
       <c r="S114" t="inlineStr">
         <is>
@@ -8644,16 +8644,16 @@
         <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>246545</v>
+        <v>246546</v>
       </c>
       <c r="P115" t="n">
         <v>548</v>
       </c>
       <c r="Q115" t="n">
-        <v>12.41973943384026</v>
+        <v>12.41974347191934</v>
       </c>
       <c r="R115" t="n">
-        <v>0.9974488677420196</v>
+        <v>0.9973945687207525</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -8714,16 +8714,16 @@
         <v>0</v>
       </c>
       <c r="O116" t="n">
-        <v>247083</v>
+        <v>247084</v>
       </c>
       <c r="P116" t="n">
         <v>121</v>
       </c>
       <c r="Q116" t="n">
-        <v>12.41846258344616</v>
+        <v>12.41846662668455</v>
       </c>
       <c r="R116" t="n">
-        <v>0.9973463218724665</v>
+        <v>0.9972920288812496</v>
       </c>
       <c r="S116" t="inlineStr">
         <is>
@@ -8783,16 +8783,16 @@
         <v>0</v>
       </c>
       <c r="O117" t="n">
-        <v>255005</v>
+        <v>255006</v>
       </c>
       <c r="P117" t="n">
         <v>111</v>
       </c>
       <c r="Q117" t="n">
-        <v>12.44991254230255</v>
+        <v>12.44991646036028</v>
       </c>
       <c r="R117" t="n">
-        <v>0.999872117684765</v>
+        <v>0.9998176763204473</v>
       </c>
       <c r="S117" t="inlineStr">
         <is>
@@ -8852,16 +8852,16 @@
         <v>0</v>
       </c>
       <c r="O118" t="n">
-        <v>254932</v>
+        <v>254933</v>
       </c>
       <c r="P118" t="n">
         <v>440</v>
       </c>
       <c r="Q118" t="n">
-        <v>12.45220198778941</v>
+        <v>12.45220589688725</v>
       </c>
       <c r="R118" t="n">
-        <v>1.000055986663723</v>
+        <v>1.000001534510641</v>
       </c>
       <c r="S118" t="inlineStr">
         <is>
@@ -8920,16 +8920,16 @@
         <v>0</v>
       </c>
       <c r="O119" t="n">
-        <v>255356</v>
+        <v>256357</v>
       </c>
       <c r="P119" t="n">
         <v>44</v>
       </c>
       <c r="Q119" t="n">
-        <v>12.45076240126537</v>
+        <v>12.4546733951134</v>
       </c>
       <c r="R119" t="n">
-        <v>0.9999403711988362</v>
+        <v>1.00019969233368</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -8988,16 +8988,16 @@
         <v>0</v>
       </c>
       <c r="O120" t="n">
-        <v>267877</v>
+        <v>267878</v>
       </c>
       <c r="P120" t="n">
         <v>178</v>
       </c>
       <c r="Q120" t="n">
-        <v>12.49961501286131</v>
+        <v>12.49961874094252</v>
       </c>
       <c r="R120" t="n">
-        <v>1.003863801507675</v>
+        <v>1.003809126290235</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -9066,7 +9066,7 @@
         <v>8.555066843844319</v>
       </c>
       <c r="R121" t="n">
-        <v>1.016812345523632</v>
+        <v>1.016766091225349</v>
       </c>
       <c r="S121" t="inlineStr">
         <is>
@@ -9126,16 +9126,16 @@
         <v>0</v>
       </c>
       <c r="O122" t="n">
-        <v>4837</v>
+        <v>4838</v>
       </c>
       <c r="P122" t="n">
         <v>80</v>
       </c>
       <c r="Q122" t="n">
-        <v>8.516793111394898</v>
+        <v>8.516993171413571</v>
       </c>
       <c r="R122" t="n">
-        <v>1.01226332160901</v>
+        <v>1.012241051292567</v>
       </c>
       <c r="S122" t="inlineStr">
         <is>
@@ -9196,16 +9196,16 @@
         <v>0</v>
       </c>
       <c r="O123" t="n">
-        <v>4469</v>
+        <v>4500</v>
       </c>
       <c r="P123" t="n">
         <v>14</v>
       </c>
       <c r="Q123" t="n">
-        <v>8.411388132519262</v>
+        <v>8.418256443556213</v>
       </c>
       <c r="R123" t="n">
-        <v>0.9997354143750032</v>
+        <v>1.000506232771992</v>
       </c>
       <c r="S123" t="inlineStr">
         <is>
@@ -9272,7 +9272,7 @@
         <v>8.340217320947035</v>
       </c>
       <c r="R124" t="n">
-        <v>0.9912764085988359</v>
+        <v>0.9912313159178843</v>
       </c>
       <c r="S124" t="inlineStr">
         <is>
@@ -9341,7 +9341,7 @@
         <v>8.464635940677562</v>
       </c>
       <c r="R125" t="n">
-        <v>1.006064181840612</v>
+        <v>1.006018416471059</v>
       </c>
       <c r="S125" t="inlineStr">
         <is>
@@ -9412,7 +9412,7 @@
         <v>6.107022887742255</v>
       </c>
       <c r="R126" t="n">
-        <v>1.027075342828327</v>
+        <v>1.027026320581074</v>
       </c>
       <c r="S126" t="inlineStr">
         <is>
@@ -9480,7 +9480,7 @@
         <v>6.030685260261263</v>
       </c>
       <c r="R127" t="n">
-        <v>1.014236927718879</v>
+        <v>1.014188518248443</v>
       </c>
       <c r="S127" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
         <v>5.924255797414532</v>
       </c>
       <c r="R128" t="n">
-        <v>0.9963376862963933</v>
+        <v>0.9962901311557251</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
@@ -9616,7 +9616,7 @@
         <v>5.808142489980444</v>
       </c>
       <c r="R129" t="n">
-        <v>0.9768098218635999</v>
+        <v>0.976763198786782</v>
       </c>
       <c r="S129" t="inlineStr">
         <is>
@@ -9684,7 +9684,7 @@
         <v>5.855071922202427</v>
       </c>
       <c r="R130" t="n">
-        <v>0.9847023848315359</v>
+        <v>0.9846553850431398</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
@@ -9752,7 +9752,7 @@
         <v>5.883322388488279</v>
       </c>
       <c r="R131" t="n">
-        <v>0.9894535308283586</v>
+        <v>0.9894063042680363</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -9820,7 +9820,7 @@
         <v>5.89440283426485</v>
       </c>
       <c r="R132" t="n">
-        <v>0.9913170333653322</v>
+        <v>0.9912697178601406</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
@@ -9888,7 +9888,7 @@
         <v>5.916202062607435</v>
       </c>
       <c r="R133" t="n">
-        <v>0.9949832141435788</v>
+        <v>0.9949357236517888</v>
       </c>
       <c r="S133" t="inlineStr">
         <is>
@@ -9956,7 +9956,7 @@
         <v>6.045005314036012</v>
       </c>
       <c r="R134" t="n">
-        <v>1.016645265530997</v>
+        <v>1.016596741110735</v>
       </c>
       <c r="S134" t="inlineStr">
         <is>
@@ -10024,7 +10024,7 @@
         <v>6.126869184114185</v>
       </c>
       <c r="R135" t="n">
-        <v>1.030413080712197</v>
+        <v>1.030363899154906</v>
       </c>
       <c r="S135" t="inlineStr">
         <is>
@@ -10092,7 +10092,7 @@
         <v>5.981414211254481</v>
       </c>
       <c r="R136" t="n">
-        <v>1.005950553084239</v>
+        <v>1.005902539121989</v>
       </c>
       <c r="S136" t="inlineStr">
         <is>
@@ -10160,7 +10160,7 @@
         <v>6.052089168924417</v>
       </c>
       <c r="R137" t="n">
-        <v>1.017836623877247</v>
+        <v>1.01778804259352</v>
       </c>
       <c r="S137" t="inlineStr">
         <is>
@@ -10219,16 +10219,16 @@
         <v>0</v>
       </c>
       <c r="O138" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="P138" t="n">
         <v>1</v>
       </c>
       <c r="Q138" t="n">
-        <v>5.968707559985366</v>
+        <v>5.971261839790462</v>
       </c>
       <c r="R138" t="n">
-        <v>1.003813556310472</v>
+        <v>1.004195201045561</v>
       </c>
       <c r="S138" t="inlineStr">
         <is>
@@ -10287,16 +10287,16 @@
         <v>0</v>
       </c>
       <c r="O139" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="P139" t="n">
         <v>4</v>
       </c>
       <c r="Q139" t="n">
-        <v>6.021023349349527</v>
+        <v>6.023447592961033</v>
       </c>
       <c r="R139" t="n">
-        <v>1.012611993500609</v>
+        <v>1.012971349923781</v>
       </c>
       <c r="S139" t="inlineStr">
         <is>
@@ -10355,16 +10355,16 @@
         <v>0</v>
       </c>
       <c r="O140" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="P140" t="n">
         <v>4</v>
       </c>
       <c r="Q140" t="n">
-        <v>5.983936280687191</v>
+        <v>5.986452005284438</v>
       </c>
       <c r="R140" t="n">
-        <v>1.006374713165976</v>
+        <v>1.006749751775608</v>
       </c>
       <c r="S140" t="inlineStr">
         <is>
@@ -10423,16 +10423,16 @@
         <v>0</v>
       </c>
       <c r="O141" t="n">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="P141" t="n">
         <v>3</v>
       </c>
       <c r="Q141" t="n">
-        <v>5.942799375126701</v>
+        <v>5.945420608606575</v>
       </c>
       <c r="R141" t="n">
-        <v>0.9994563337594996</v>
+        <v>0.9998494461548528</v>
       </c>
       <c r="S141" t="inlineStr">
         <is>
@@ -10500,7 +10500,7 @@
         <v>5.983936280687191</v>
       </c>
       <c r="R142" t="n">
-        <v>1.006374713165976</v>
+        <v>1.006326678958591</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -10568,7 +10568,7 @@
         <v>5.87493073085203</v>
       </c>
       <c r="R143" t="n">
-        <v>0.9880422270225473</v>
+        <v>0.9879950678236747</v>
       </c>
       <c r="S143" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         <v>5.905361848054571</v>
       </c>
       <c r="R144" t="n">
-        <v>0.9931601135456487</v>
+        <v>0.9931127100703457</v>
       </c>
       <c r="S144" t="inlineStr">
         <is>
@@ -10704,7 +10704,7 @@
         <v>5.886104031450156</v>
       </c>
       <c r="R145" t="n">
-        <v>0.9899213458261426</v>
+        <v>0.9898740969370373</v>
       </c>
       <c r="S145" t="inlineStr">
         <is>
@@ -10772,7 +10772,7 @@
         <v>5.857933154483459</v>
       </c>
       <c r="R146" t="n">
-        <v>0.9851835851119296</v>
+        <v>0.9851365623558717</v>
       </c>
       <c r="S146" t="inlineStr">
         <is>
@@ -10840,7 +10840,7 @@
         <v>5.852202479774474</v>
       </c>
       <c r="R147" t="n">
-        <v>0.9842198037736966</v>
+        <v>0.9841728270188668</v>
       </c>
       <c r="S147" t="inlineStr">
         <is>
@@ -10908,7 +10908,7 @@
         <v>5.84354441703136</v>
       </c>
       <c r="R148" t="n">
-        <v>0.9827636961213146</v>
+        <v>0.9827167888664196</v>
       </c>
       <c r="S148" t="inlineStr">
         <is>
@@ -10976,7 +10976,7 @@
         <v>5.921578419643816</v>
       </c>
       <c r="R149" t="n">
-        <v>0.9958874065541544</v>
+        <v>0.9958398729053125</v>
       </c>
       <c r="S149" t="inlineStr">
         <is>
@@ -11044,7 +11044,7 @@
         <v>5.940171252720432</v>
       </c>
       <c r="R150" t="n">
-        <v>0.9990143377540758</v>
+        <v>0.9989666548569869</v>
       </c>
       <c r="S150" t="inlineStr">
         <is>
@@ -11112,7 +11112,7 @@
         <v>6.021023349349527</v>
       </c>
       <c r="R151" t="n">
-        <v>1.012611993500609</v>
+        <v>1.01256366158819</v>
       </c>
       <c r="S151" t="inlineStr">
         <is>
@@ -11180,7 +11180,7 @@
         <v>5.971261839790462</v>
       </c>
       <c r="R152" t="n">
-        <v>1.004243133512772</v>
+        <v>1.004195201045561</v>
       </c>
       <c r="S152" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
         <v>5.996452088619021</v>
       </c>
       <c r="R153" t="n">
-        <v>1.008479614024979</v>
+        <v>1.008431479350796</v>
       </c>
       <c r="S153" t="inlineStr">
         <is>
@@ -11316,7 +11316,7 @@
         <v>6.054439346269371</v>
       </c>
       <c r="R154" t="n">
-        <v>1.018231875253678</v>
+        <v>1.018183275104626</v>
       </c>
       <c r="S154" t="inlineStr">
         <is>
@@ -11384,7 +11384,7 @@
         <v>6.084499413075172</v>
       </c>
       <c r="R155" t="n">
-        <v>1.023287358749897</v>
+        <v>1.023238517302907</v>
       </c>
       <c r="S155" t="inlineStr">
         <is>
@@ -11457,7 +11457,7 @@
         <v>0.176</v>
       </c>
       <c r="E2" t="n">
-        <v>142.296</v>
+        <v>142.302</v>
       </c>
       <c r="F2" t="n">
         <v>33.3</v>
@@ -11567,7 +11567,7 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>30.561</v>
+        <v>30.567</v>
       </c>
       <c r="F7" t="n">
         <v>5.9</v>
@@ -11633,7 +11633,7 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>9.727</v>
+        <v>9.728999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>

</xml_diff>